<commit_message>
Clean up code comments and update RouteSchedule.xls
</commit_message>
<xml_diff>
--- a/RouteSchedule.xlsx
+++ b/RouteSchedule.xlsx
@@ -8,66 +8,67 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marshallhuckins/Desktop/AMS Routes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4E8DCB2-55F5-FB4F-B7B4-8E89F33E2F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B746405-D7C1-B441-8B95-24CEFA666586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15880" yWindow="860" windowWidth="34200" windowHeight="21460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="21_URBANDALE" sheetId="42" r:id="rId1"/>
     <sheet name="32_Route1" sheetId="52" r:id="rId2"/>
-    <sheet name="47_CedarRapids" sheetId="49" r:id="rId3"/>
-    <sheet name="51_AM_EAST" sheetId="41" r:id="rId4"/>
-    <sheet name="51_AM_NORTH" sheetId="38" r:id="rId5"/>
-    <sheet name="51_AM_SOUTH" sheetId="40" r:id="rId6"/>
-    <sheet name="51_AM_WEST" sheetId="12" r:id="rId7"/>
-    <sheet name="51_NT_1" sheetId="44" r:id="rId8"/>
-    <sheet name="51_NT_2" sheetId="45" r:id="rId9"/>
-    <sheet name="51_NT_3" sheetId="46" r:id="rId10"/>
-    <sheet name="51_NT_4" sheetId="47" r:id="rId11"/>
-    <sheet name="51_NT_5" sheetId="48" r:id="rId12"/>
-    <sheet name="51_PM_NORTH" sheetId="39" r:id="rId13"/>
-    <sheet name="51_PM_WEST" sheetId="13" r:id="rId14"/>
-    <sheet name="51_SATURDAY" sheetId="43" r:id="rId15"/>
-    <sheet name="52_Route1" sheetId="50" r:id="rId16"/>
-    <sheet name="52_Route2" sheetId="51" r:id="rId17"/>
-    <sheet name="52_Route3" sheetId="53" r:id="rId18"/>
-    <sheet name="52_Route4" sheetId="54" r:id="rId19"/>
-    <sheet name="52_Route5" sheetId="55" r:id="rId20"/>
-    <sheet name="60_64" sheetId="10" r:id="rId21"/>
-    <sheet name="60_64_B" sheetId="24" r:id="rId22"/>
-    <sheet name="60_ATLANTIC_SHUTTLE" sheetId="11" r:id="rId23"/>
-    <sheet name="60_BELLEVUE_GLENWOOD_EVEN" sheetId="7" r:id="rId24"/>
-    <sheet name="60_BELLEVUE_GLENWOOD_ODD" sheetId="8" r:id="rId25"/>
-    <sheet name="60_CB_CORN_EVEN" sheetId="5" r:id="rId26"/>
-    <sheet name="60_CB_CORN_ODD" sheetId="6" r:id="rId27"/>
-    <sheet name="60_GRAND_ISLAND_MIDDAY" sheetId="32" r:id="rId28"/>
-    <sheet name="60_GRAND_ISLAND_NT" sheetId="33" r:id="rId29"/>
-    <sheet name="60_LINCOLN_MIDDAY" sheetId="30" r:id="rId30"/>
-    <sheet name="60_MISSOURI_EAST_NT" sheetId="35" r:id="rId31"/>
-    <sheet name="60_NORTH_MIDDAY_73_68_78" sheetId="31" r:id="rId32"/>
-    <sheet name="60_RED_NT" sheetId="34" r:id="rId33"/>
-    <sheet name="60_SIOUXCITY_MIDDAY" sheetId="9" r:id="rId34"/>
-    <sheet name="60_WEST_NT" sheetId="36" r:id="rId35"/>
-    <sheet name="66_67_69_MEETUP_FAIRBURY" sheetId="57" r:id="rId36"/>
-    <sheet name="66_67_69_MEETUP_GENEVA" sheetId="58" r:id="rId37"/>
-    <sheet name="66_67_69_MIDDAY_MEETUP" sheetId="56" r:id="rId38"/>
-    <sheet name="83_EM_North" sheetId="26" r:id="rId39"/>
-    <sheet name="83_EM_SOUTH" sheetId="27" r:id="rId40"/>
-    <sheet name="83_LM" sheetId="29" r:id="rId41"/>
-    <sheet name="83_NT" sheetId="28" r:id="rId42"/>
-    <sheet name="BR30_1" sheetId="1" r:id="rId43"/>
-    <sheet name="BR30_2" sheetId="2" r:id="rId44"/>
-    <sheet name="BR30_3" sheetId="3" r:id="rId45"/>
-    <sheet name="BR30_4" sheetId="4" r:id="rId46"/>
-    <sheet name="BR30_Night_A" sheetId="18" r:id="rId47"/>
-    <sheet name="BR30_Night_B" sheetId="19" r:id="rId48"/>
-    <sheet name="BR30_Night_C" sheetId="20" r:id="rId49"/>
-    <sheet name="BR30_Night_D" sheetId="21" r:id="rId50"/>
-    <sheet name="BR30_Night_E" sheetId="22" r:id="rId51"/>
+    <sheet name="43_Merrill" sheetId="59" r:id="rId3"/>
+    <sheet name="47_CedarRapids" sheetId="49" r:id="rId4"/>
+    <sheet name="51_AM_EAST" sheetId="41" r:id="rId5"/>
+    <sheet name="51_AM_NORTH" sheetId="38" r:id="rId6"/>
+    <sheet name="51_AM_SOUTH" sheetId="40" r:id="rId7"/>
+    <sheet name="51_AM_WEST" sheetId="12" r:id="rId8"/>
+    <sheet name="51_NT_1" sheetId="44" r:id="rId9"/>
+    <sheet name="51_NT_2" sheetId="45" r:id="rId10"/>
+    <sheet name="51_NT_3" sheetId="46" r:id="rId11"/>
+    <sheet name="51_NT_4" sheetId="47" r:id="rId12"/>
+    <sheet name="51_NT_5" sheetId="48" r:id="rId13"/>
+    <sheet name="51_PM_NORTH" sheetId="39" r:id="rId14"/>
+    <sheet name="51_PM_WEST" sheetId="13" r:id="rId15"/>
+    <sheet name="51_SATURDAY" sheetId="43" r:id="rId16"/>
+    <sheet name="52_Route1" sheetId="50" r:id="rId17"/>
+    <sheet name="52_Route2" sheetId="51" r:id="rId18"/>
+    <sheet name="52_Route3" sheetId="53" r:id="rId19"/>
+    <sheet name="52_Route4" sheetId="54" r:id="rId20"/>
+    <sheet name="52_Route5" sheetId="55" r:id="rId21"/>
+    <sheet name="60_64" sheetId="10" r:id="rId22"/>
+    <sheet name="60_64_B" sheetId="24" r:id="rId23"/>
+    <sheet name="60_ATLANTIC_SHUTTLE" sheetId="11" r:id="rId24"/>
+    <sheet name="60_BELLEVUE_GLENWOOD_EVEN" sheetId="7" r:id="rId25"/>
+    <sheet name="60_BELLEVUE_GLENWOOD_ODD" sheetId="8" r:id="rId26"/>
+    <sheet name="60_CB_CORN_EVEN" sheetId="5" r:id="rId27"/>
+    <sheet name="60_CB_CORN_ODD" sheetId="6" r:id="rId28"/>
+    <sheet name="60_GRAND_ISLAND_MIDDAY" sheetId="32" r:id="rId29"/>
+    <sheet name="60_GRAND_ISLAND_NT" sheetId="33" r:id="rId30"/>
+    <sheet name="60_LINCOLN_MIDDAY" sheetId="30" r:id="rId31"/>
+    <sheet name="60_MISSOURI_EAST_NT" sheetId="35" r:id="rId32"/>
+    <sheet name="60_NORTH_MIDDAY_73_68_78" sheetId="31" r:id="rId33"/>
+    <sheet name="60_RED_NT" sheetId="34" r:id="rId34"/>
+    <sheet name="60_SIOUXCITY_MIDDAY" sheetId="9" r:id="rId35"/>
+    <sheet name="60_WEST_NT" sheetId="36" r:id="rId36"/>
+    <sheet name="66_67_69_MEETUP_FAIRBURY" sheetId="57" r:id="rId37"/>
+    <sheet name="66_67_69_MEETUP_GENEVA" sheetId="58" r:id="rId38"/>
+    <sheet name="66_67_69_MIDDAY_MEETUP" sheetId="56" r:id="rId39"/>
+    <sheet name="83_EM_North" sheetId="26" r:id="rId40"/>
+    <sheet name="83_EM_SOUTH" sheetId="27" r:id="rId41"/>
+    <sheet name="83_LM" sheetId="29" r:id="rId42"/>
+    <sheet name="83_NT" sheetId="28" r:id="rId43"/>
+    <sheet name="BR30_1" sheetId="1" r:id="rId44"/>
+    <sheet name="BR30_2" sheetId="2" r:id="rId45"/>
+    <sheet name="BR30_3" sheetId="3" r:id="rId46"/>
+    <sheet name="BR30_4" sheetId="4" r:id="rId47"/>
+    <sheet name="BR30_Night_A" sheetId="18" r:id="rId48"/>
+    <sheet name="BR30_Night_B" sheetId="19" r:id="rId49"/>
+    <sheet name="BR30_Night_C" sheetId="20" r:id="rId50"/>
+    <sheet name="BR30_Night_D" sheetId="21" r:id="rId51"/>
+    <sheet name="BR30_Night_E" sheetId="22" r:id="rId52"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="36" hidden="1">'66_67_69_MEETUP_GENEVA'!$A$1:$H$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="47" hidden="1">BR30_Night_B!$G$2:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="37" hidden="1">'66_67_69_MEETUP_GENEVA'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="48" hidden="1">BR30_Night_B!$G$2:$G$10</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -86,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1529" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="163">
   <si>
     <t>Trip_ID</t>
   </si>
@@ -569,6 +570,12 @@
   </si>
   <si>
     <t>BR56</t>
+  </si>
+  <si>
+    <t>43_Merrill</t>
+  </si>
+  <si>
+    <t>BR43</t>
   </si>
 </sst>
 </file>
@@ -1148,6 +1155,152 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EBCC13C-AA15-7440-B91A-5770844563BE}">
+  <sheetPr codeName="Sheet48"/>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>133</v>
+      </c>
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.27083333333333331</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7DE4201-C3DB-DC47-B443-C82ACE93B339}">
   <sheetPr codeName="Sheet49"/>
   <dimension ref="A1:H6"/>
@@ -1275,7 +1428,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3D22B2B-C481-9A41-B931-DCC76B320ECF}">
   <sheetPr codeName="Sheet50"/>
   <dimension ref="A1:H10"/>
@@ -1481,7 +1634,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{253D3D8D-4543-B046-9D23-0062E7084B6E}">
   <sheetPr codeName="Sheet51"/>
   <dimension ref="A1:H5"/>
@@ -1583,7 +1736,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE7B4EA8-5BC0-2648-BD0E-4B668490B784}">
   <sheetPr codeName="Sheet24"/>
   <dimension ref="A1:H7"/>
@@ -1731,7 +1884,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{100D656A-C838-364D-8F00-92D41823B05F}">
   <sheetPr codeName="Sheet21"/>
   <dimension ref="A1:G5"/>
@@ -1854,7 +2007,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D90D93F-F95F-8D46-BC35-0BD63B7FB098}">
   <sheetPr codeName="Sheet28"/>
   <dimension ref="A1:H6"/>
@@ -1985,7 +2138,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F214C945-893C-614D-A9F1-86C7995CEA1B}">
   <sheetPr codeName="Sheet29"/>
   <dimension ref="A1:H8"/>
@@ -2156,7 +2309,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4925C1E5-977F-8641-92D0-FC7DDDE2436A}">
   <sheetPr codeName="Sheet30"/>
   <dimension ref="A1:H7"/>
@@ -2307,7 +2460,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5387C99-5097-BA43-952A-89AAB0D63D27}">
   <sheetPr codeName="Sheet44"/>
   <dimension ref="A1:H7"/>
@@ -2445,157 +2598,6 @@
       </c>
       <c r="C7" s="2">
         <v>0.60763888888888884</v>
-      </c>
-      <c r="E7">
-        <v>6</v>
-      </c>
-      <c r="F7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5568A20A-6FE2-4F4E-8740-15520BFC133E}">
-  <sheetPr codeName="Sheet45"/>
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B2" t="s">
-        <v>141</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.3263888888888889</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>154</v>
-      </c>
-      <c r="B3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.33680555555555558</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.34027777777777779</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>154</v>
-      </c>
-      <c r="B4" t="s">
-        <v>141</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.35069444444444442</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0.36805555555555558</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>154</v>
-      </c>
-      <c r="B5" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0.37847222222222221</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0.38194444444444442</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>154</v>
-      </c>
-      <c r="B6" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0.3923611111111111</v>
-      </c>
-      <c r="D6" s="2">
-        <v>0.4236111111111111</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>154</v>
-      </c>
-      <c r="B7" t="s">
-        <v>140</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0.43402777777777779</v>
       </c>
       <c r="E7">
         <v>6</v>
@@ -2741,6 +2743,157 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5568A20A-6FE2-4F4E-8740-15520BFC133E}">
+  <sheetPr codeName="Sheet45"/>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.3263888888888889</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.33680555555555558</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.34027777777777779</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.36805555555555558</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>154</v>
+      </c>
+      <c r="B5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.37847222222222221</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.38194444444444442</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>154</v>
+      </c>
+      <c r="B6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.3923611111111111</v>
+      </c>
+      <c r="D6" s="2">
+        <v>0.4236111111111111</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>154</v>
+      </c>
+      <c r="B7" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.43402777777777779</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B8FA4C-B3CB-114C-9531-298AD4A8696E}">
   <sheetPr codeName="Sheet46"/>
   <dimension ref="A1:H14"/>
@@ -3032,7 +3185,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E916533-040C-F74A-848A-305F4573B66B}">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:G4"/>
@@ -3129,7 +3282,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29B98485-1BEC-9A4E-AEDA-1001166E85E7}">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:G4"/>
@@ -3229,7 +3382,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49763124-1699-7D4B-B9EF-92F40DAC1909}">
   <sheetPr codeName="Sheet12"/>
   <dimension ref="A1:G6"/>
@@ -3373,7 +3526,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76C3F466-EEC1-6548-8F82-093A399C5022}">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:G11"/>
@@ -3631,7 +3784,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E38B432-80D0-084C-9C24-9561C3C327AE}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:G14"/>
@@ -3961,7 +4114,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FB1D438-269D-6344-AAB6-4CB84A923FB3}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:G17"/>
@@ -4361,7 +4514,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F9F8785-C8CF-1945-8D60-2C2B7B8C18E0}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:G17"/>
@@ -4703,7 +4856,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7F1648B-214D-7548-97EE-C5E9970A9FC3}">
   <sheetPr codeName="Sheet14"/>
   <dimension ref="A1:G7"/>
@@ -4872,7 +5025,138 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5110ACEC-7611-5B40-B763-07E9A982B216}">
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.43055555555555558</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B4" t="s">
+        <v>162</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.44097222222222221</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>161</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.67708333333333337</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.68055555555555558</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>161</v>
+      </c>
+      <c r="B6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.6875</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC3254C4-E8BB-CA4C-8E9A-3A2CF48FD7C2}">
   <sheetPr codeName="Sheet15"/>
   <dimension ref="A1:G5"/>
@@ -4980,7 +5264,1139 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{885BC41D-4C36-884F-B715-968C4CD5CB72}">
+  <sheetPr codeName="Sheet19"/>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.37152777777777779</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.41319444444444442</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.46875</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.49652777777777779</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.53819444444444442</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.59375</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C7BB505-331C-7F4C-BAE9-1BDF4EDE982F}">
+  <sheetPr codeName="Sheet17"/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.14583333333333334</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1187C91-8616-9745-98C9-DCF5A12305EF}">
+  <sheetPr codeName="Sheet13"/>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.46875</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.53125</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.57986111111111116</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.61111111111111116</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.6875</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3992E15C-8544-A94D-B443-1EA62C6EB477}">
+  <sheetPr codeName="Sheet16"/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5654A771-B573-A542-AE3A-EDA834F02BFC}">
+  <sheetPr codeName="Sheet11"/>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.47222222222222221</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.56944444444444442</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.67708333333333337</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA06B990-1EE7-0B4E-8B60-63D05407C907}">
+  <sheetPr codeName="Sheet18"/>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" t="s">
+        <v>106</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" t="s">
+        <v>77</v>
+      </c>
+      <c r="E8">
+        <v>7</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="E9">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D91A9337-13C8-D940-AAD9-27793377CCE0}">
+  <sheetPr codeName="Sheet42"/>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="24.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.58680555555555558</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>158</v>
+      </c>
+      <c r="B4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC2FBC46-1C89-7141-9F98-8B3E8DDF3228}">
+  <sheetPr codeName="Sheet41"/>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.58680555555555558</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62968357-C14C-7A44-A92C-6AE15D6EE140}">
+  <sheetPr codeName="Sheet31"/>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.58680555555555558</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFA2DB04-608A-D64B-AA09-79759688C227}">
   <sheetPr codeName="Sheet22"/>
   <dimension ref="A1:H4"/>
@@ -5074,1139 +6490,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{885BC41D-4C36-884F-B715-968C4CD5CB72}">
-  <sheetPr codeName="Sheet19"/>
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="12" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.37152777777777779</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.41319444444444442</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.46875</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0.49652777777777779</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0.53819444444444442</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0.59375</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C7BB505-331C-7F4C-BAE9-1BDF4EDE982F}">
-  <sheetPr codeName="Sheet17"/>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="12" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>103</v>
-      </c>
-      <c r="B5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B6" t="s">
-        <v>46</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>103</v>
-      </c>
-      <c r="B7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0.14583333333333334</v>
-      </c>
-      <c r="E7">
-        <v>6</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1187C91-8616-9745-98C9-DCF5A12305EF}">
-  <sheetPr codeName="Sheet13"/>
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="H1" s="13" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.46875</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.52083333333333337</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.53125</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>95</v>
-      </c>
-      <c r="B4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.57291666666666663</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0.57986111111111116</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0.61111111111111116</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" t="s">
-        <v>76</v>
-      </c>
-      <c r="H5" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>97</v>
-      </c>
-      <c r="B6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0.6875</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3992E15C-8544-A94D-B443-1EA62C6EB477}">
-  <sheetPr codeName="Sheet16"/>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="12" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B3" t="s">
-        <v>90</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B4" t="s">
-        <v>91</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>101</v>
-      </c>
-      <c r="B5" t="s">
-        <v>102</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>101</v>
-      </c>
-      <c r="B6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>101</v>
-      </c>
-      <c r="B7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0.25</v>
-      </c>
-      <c r="E7">
-        <v>6</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5654A771-B573-A542-AE3A-EDA834F02BFC}">
-  <sheetPr codeName="Sheet11"/>
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.47222222222222221</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>87</v>
-      </c>
-      <c r="B3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.56944444444444442</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.57291666666666663</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.67708333333333337</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA06B990-1EE7-0B4E-8B60-63D05407C907}">
-  <sheetPr codeName="Sheet18"/>
-  <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="12" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>104</v>
-      </c>
-      <c r="B2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>104</v>
-      </c>
-      <c r="B3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" t="s">
-        <v>105</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B5" t="s">
-        <v>106</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>104</v>
-      </c>
-      <c r="B6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>104</v>
-      </c>
-      <c r="B7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E7">
-        <v>6</v>
-      </c>
-      <c r="F7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>104</v>
-      </c>
-      <c r="B8" t="s">
-        <v>77</v>
-      </c>
-      <c r="E8">
-        <v>7</v>
-      </c>
-      <c r="F8" t="s">
-        <v>9</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>104</v>
-      </c>
-      <c r="B9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C9" s="2">
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="E9">
-        <v>8</v>
-      </c>
-      <c r="F9" t="s">
-        <v>9</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D91A9337-13C8-D940-AAD9-27793377CCE0}">
-  <sheetPr codeName="Sheet42"/>
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="24.33203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>158</v>
-      </c>
-      <c r="B2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>158</v>
-      </c>
-      <c r="B3" t="s">
-        <v>157</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.58680555555555558</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>158</v>
-      </c>
-      <c r="B4" t="s">
-        <v>105</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.625</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC2FBC46-1C89-7141-9F98-8B3E8DDF3228}">
-  <sheetPr codeName="Sheet41"/>
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>159</v>
-      </c>
-      <c r="B2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>159</v>
-      </c>
-      <c r="B3" t="s">
-        <v>157</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.58680555555555558</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>159</v>
-      </c>
-      <c r="B4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.625</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62968357-C14C-7A44-A92C-6AE15D6EE140}">
-  <sheetPr codeName="Sheet31"/>
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="23.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>156</v>
-      </c>
-      <c r="B2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>156</v>
-      </c>
-      <c r="B3" t="s">
-        <v>157</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.58680555555555558</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.625</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{538A7D11-9BEC-DE43-B110-52E6248351DE}">
   <sheetPr codeName="Sheet37"/>
   <dimension ref="A1:G5"/>
@@ -6329,178 +6613,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4F36657-4F49-CA45-B09B-4FCCD08126E8}">
-  <sheetPr codeName="Sheet26"/>
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>123</v>
-      </c>
-      <c r="B2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.45833333333333331</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>123</v>
-      </c>
-      <c r="B3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.4826388888888889</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.4861111111111111</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.52777777777777779</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0.53125</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0.5625</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0.56597222222222221</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>123</v>
-      </c>
-      <c r="B6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0.59722222222222221</v>
-      </c>
-      <c r="D6" s="2">
-        <v>0.60069444444444442</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>123</v>
-      </c>
-      <c r="B7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0.61458333333333337</v>
-      </c>
-      <c r="D7" s="2">
-        <v>0.61805555555555558</v>
-      </c>
-      <c r="E7">
-        <v>6</v>
-      </c>
-      <c r="F7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>123</v>
-      </c>
-      <c r="B8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C8" s="2">
-        <v>0.67708333333333337</v>
-      </c>
-      <c r="E8">
-        <v>7</v>
-      </c>
-      <c r="F8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{216DADC4-5F76-6D4D-AA35-839615F53477}">
   <sheetPr codeName="Sheet38"/>
   <dimension ref="A1:G6"/>
@@ -6643,7 +6756,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE22F097-E2E5-874D-8EDF-90425A618917}">
   <sheetPr codeName="Sheet40"/>
   <dimension ref="A1:G5"/>
@@ -6765,7 +6878,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F353A1C7-62FC-C84A-BDFD-003B4C4A7713}">
   <sheetPr codeName="Sheet39"/>
   <dimension ref="A1:G7"/>
@@ -6932,7 +7045,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:G6"/>
@@ -7065,7 +7178,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:G5"/>
@@ -7173,7 +7286,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E95C35C-82EF-AE4F-9BDF-8EDBBC469555}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:G7"/>
@@ -7321,7 +7434,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E6EA992-E3C6-294E-89AC-5B22FDC208AB}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:G9"/>
@@ -7535,7 +7648,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEA0C3CF-67BD-3F46-B5EA-05756EEE6C40}">
   <sheetPr codeName="Sheet32"/>
   <dimension ref="A1:G7"/>
@@ -7677,7 +7790,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9F2857C-EA9E-CB49-9CF8-07047A99E53B}">
   <sheetPr codeName="Sheet33"/>
   <dimension ref="A1:G10"/>
@@ -7874,7 +7987,178 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4F36657-4F49-CA45-B09B-4FCCD08126E8}">
+  <sheetPr codeName="Sheet26"/>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.4826388888888889</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.4861111111111111</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.52777777777777779</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.53125</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.5625</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.56597222222222221</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.59722222222222221</v>
+      </c>
+      <c r="D6" s="2">
+        <v>0.60069444444444442</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0.61805555555555558</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0.67708333333333337</v>
+      </c>
+      <c r="E8">
+        <v>7</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{422AE880-0C69-104F-AA9B-DA4856BD7616}">
   <sheetPr codeName="Sheet34"/>
   <dimension ref="A1:G11"/>
@@ -8085,141 +8369,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DEAC3F7-93EC-9C40-A8D3-54A6AEC6A859}">
-  <sheetPr codeName="Sheet23"/>
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.39583333333333331</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>117</v>
-      </c>
-      <c r="B3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.41319444444444442</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>117</v>
-      </c>
-      <c r="B4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.44097222222222221</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0.44444444444444442</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-      <c r="H4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0.46180555555555558</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0.46527777777777779</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>117</v>
-      </c>
-      <c r="B6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46399228-8395-7647-B644-8C049B767FB1}">
   <sheetPr codeName="Sheet35"/>
   <dimension ref="A1:G6"/>
@@ -8347,7 +8497,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DB5B155-5FF2-2144-9081-38DF5FF7C409}">
   <sheetPr codeName="Sheet36"/>
   <dimension ref="A1:G7"/>
@@ -8493,6 +8643,140 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DEAC3F7-93EC-9C40-A8D3-54A6AEC6A859}">
+  <sheetPr codeName="Sheet23"/>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.41319444444444442</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.44097222222222221</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.46180555555555558</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.46527777777777779</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2F54CC2-D6D1-BE46-B16D-153B8C00D214}">
   <sheetPr codeName="Sheet25"/>
   <dimension ref="A1:H8"/>
@@ -8648,7 +8932,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20568EDA-179F-1C44-ABA9-5A9A58C75F1D}">
   <sheetPr codeName="Sheet20"/>
   <dimension ref="A1:G6"/>
@@ -8795,7 +9079,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C2CEFD-0A5C-4C44-8C30-48C59FA8DD76}">
   <sheetPr codeName="Sheet47"/>
   <dimension ref="A1:H8"/>
@@ -8956,150 +9240,4 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EBCC13C-AA15-7440-B91A-5770844563BE}">
-  <sheetPr codeName="Sheet48"/>
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>133</v>
-      </c>
-      <c r="B2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.75</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>133</v>
-      </c>
-      <c r="B3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>133</v>
-      </c>
-      <c r="B4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>133</v>
-      </c>
-      <c r="B5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>133</v>
-      </c>
-      <c r="B6" t="s">
-        <v>49</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>133</v>
-      </c>
-      <c r="B7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0.27083333333333331</v>
-      </c>
-      <c r="E7">
-        <v>6</v>
-      </c>
-      <c r="F7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add BR30 and BR60 night meetup routing
</commit_message>
<xml_diff>
--- a/RouteSchedule.xlsx
+++ b/RouteSchedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marshallhuckins/Desktop/AMS Routes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B746405-D7C1-B441-8B95-24CEFA666586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{986F3D63-79BD-6E45-B6A8-E239CDFADA0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15880" yWindow="860" windowWidth="34200" windowHeight="21460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20" yWindow="680" windowWidth="34200" windowHeight="21460" firstSheet="34" activeTab="36" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="21_URBANDALE" sheetId="42" r:id="rId1"/>
@@ -49,26 +49,28 @@
     <sheet name="60_RED_NT" sheetId="34" r:id="rId34"/>
     <sheet name="60_SIOUXCITY_MIDDAY" sheetId="9" r:id="rId35"/>
     <sheet name="60_WEST_NT" sheetId="36" r:id="rId36"/>
-    <sheet name="66_67_69_MEETUP_FAIRBURY" sheetId="57" r:id="rId37"/>
-    <sheet name="66_67_69_MEETUP_GENEVA" sheetId="58" r:id="rId38"/>
-    <sheet name="66_67_69_MIDDAY_MEETUP" sheetId="56" r:id="rId39"/>
-    <sheet name="83_EM_North" sheetId="26" r:id="rId40"/>
-    <sheet name="83_EM_SOUTH" sheetId="27" r:id="rId41"/>
-    <sheet name="83_LM" sheetId="29" r:id="rId42"/>
-    <sheet name="83_NT" sheetId="28" r:id="rId43"/>
-    <sheet name="BR30_1" sheetId="1" r:id="rId44"/>
-    <sheet name="BR30_2" sheetId="2" r:id="rId45"/>
-    <sheet name="BR30_3" sheetId="3" r:id="rId46"/>
-    <sheet name="BR30_4" sheetId="4" r:id="rId47"/>
-    <sheet name="BR30_Night_A" sheetId="18" r:id="rId48"/>
-    <sheet name="BR30_Night_B" sheetId="19" r:id="rId49"/>
-    <sheet name="BR30_Night_C" sheetId="20" r:id="rId50"/>
-    <sheet name="BR30_Night_D" sheetId="21" r:id="rId51"/>
-    <sheet name="BR30_Night_E" sheetId="22" r:id="rId52"/>
+    <sheet name="60_30_NT_MEETUP" sheetId="60" r:id="rId37"/>
+    <sheet name="66_67_69_MEETUP_FAIRBURY" sheetId="57" r:id="rId38"/>
+    <sheet name="66_67_69_MEETUP_GENEVA" sheetId="58" r:id="rId39"/>
+    <sheet name="66_67_69_MIDDAY_MEETUP" sheetId="56" r:id="rId40"/>
+    <sheet name="83_EM_North" sheetId="26" r:id="rId41"/>
+    <sheet name="83_EM_SOUTH" sheetId="27" r:id="rId42"/>
+    <sheet name="83_LM" sheetId="29" r:id="rId43"/>
+    <sheet name="83_NT" sheetId="28" r:id="rId44"/>
+    <sheet name="BR30_1" sheetId="1" r:id="rId45"/>
+    <sheet name="BR30_2" sheetId="2" r:id="rId46"/>
+    <sheet name="BR30_3" sheetId="3" r:id="rId47"/>
+    <sheet name="BR30_4" sheetId="4" r:id="rId48"/>
+    <sheet name="BR30_Night_A" sheetId="18" r:id="rId49"/>
+    <sheet name="BR30_Night_B" sheetId="19" r:id="rId50"/>
+    <sheet name="BR30_Night_C" sheetId="20" r:id="rId51"/>
+    <sheet name="BR30_Night_D" sheetId="21" r:id="rId52"/>
+    <sheet name="BR30_Night_E" sheetId="22" r:id="rId53"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="37" hidden="1">'66_67_69_MEETUP_GENEVA'!$A$1:$H$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="48" hidden="1">BR30_Night_B!$G$2:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="36" hidden="1">'60_30_NT_MEETUP'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="38" hidden="1">'66_67_69_MEETUP_GENEVA'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="49" hidden="1">BR30_Night_B!$G$2:$G$10</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -87,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1571" uniqueCount="164">
   <si>
     <t>Trip_ID</t>
   </si>
@@ -576,6 +578,9 @@
   </si>
   <si>
     <t>BR43</t>
+  </si>
+  <si>
+    <t>60_30_NT_MEETUP</t>
   </si>
 </sst>
 </file>
@@ -6115,6 +6120,105 @@
 </file>
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7870511C-45AF-2D4F-AA72-76C8D8D50DBD}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.72222222222222221</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.92708333333333337</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.93402777777777779</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="2">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D91A9337-13C8-D940-AAD9-27793377CCE0}">
   <sheetPr codeName="Sheet42"/>
   <dimension ref="A1:H4"/>
@@ -6208,7 +6312,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC2FBC46-1C89-7141-9F98-8B3E8DDF3228}">
   <sheetPr codeName="Sheet41"/>
   <dimension ref="A1:H4"/>
@@ -6286,100 +6390,6 @@
       </c>
       <c r="B4" t="s">
         <v>106</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.625</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62968357-C14C-7A44-A92C-6AE15D6EE140}">
-  <sheetPr codeName="Sheet31"/>
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="23.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>156</v>
-      </c>
-      <c r="B2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>156</v>
-      </c>
-      <c r="B3" t="s">
-        <v>157</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.58680555555555558</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B4" t="s">
-        <v>86</v>
       </c>
       <c r="C4" s="2">
         <v>0.625</v>
@@ -6491,6 +6501,100 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62968357-C14C-7A44-A92C-6AE15D6EE140}">
+  <sheetPr codeName="Sheet31"/>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.58680555555555558</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{538A7D11-9BEC-DE43-B110-52E6248351DE}">
   <sheetPr codeName="Sheet37"/>
   <dimension ref="A1:G5"/>
@@ -6613,7 +6717,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{216DADC4-5F76-6D4D-AA35-839615F53477}">
   <sheetPr codeName="Sheet38"/>
   <dimension ref="A1:G6"/>
@@ -6756,7 +6860,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE22F097-E2E5-874D-8EDF-90425A618917}">
   <sheetPr codeName="Sheet40"/>
   <dimension ref="A1:G5"/>
@@ -6878,7 +6982,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F353A1C7-62FC-C84A-BDFD-003B4C4A7713}">
   <sheetPr codeName="Sheet39"/>
   <dimension ref="A1:G7"/>
@@ -7045,7 +7149,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:G6"/>
@@ -7178,7 +7282,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:G5"/>
@@ -7286,7 +7390,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E95C35C-82EF-AE4F-9BDF-8EDBBC469555}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:G7"/>
@@ -7434,7 +7538,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E6EA992-E3C6-294E-89AC-5B22FDC208AB}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:G9"/>
@@ -7648,7 +7752,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEA0C3CF-67BD-3F46-B5EA-05756EEE6C40}">
   <sheetPr codeName="Sheet32"/>
   <dimension ref="A1:G7"/>
@@ -7786,203 +7890,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9F2857C-EA9E-CB49-9CF8-07047A99E53B}">
-  <sheetPr codeName="Sheet33"/>
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B5" t="s">
-        <v>56</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" t="s">
-        <v>58</v>
-      </c>
-      <c r="E7">
-        <v>6</v>
-      </c>
-      <c r="F7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>55</v>
-      </c>
-      <c r="B8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8">
-        <v>7</v>
-      </c>
-      <c r="F8" t="s">
-        <v>9</v>
-      </c>
-      <c r="G8" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B9" t="s">
-        <v>60</v>
-      </c>
-      <c r="E9">
-        <v>8</v>
-      </c>
-      <c r="F9" t="s">
-        <v>9</v>
-      </c>
-      <c r="G9" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="E10">
-        <v>9</v>
-      </c>
-      <c r="F10" t="s">
-        <v>9</v>
-      </c>
-      <c r="G10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="G2:G10" xr:uid="{D9F2857C-EA9E-CB49-9CF8-07047A99E53B}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -8159,10 +8066,210 @@
 </file>
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9F2857C-EA9E-CB49-9CF8-07047A99E53B}">
+  <sheetPr codeName="Sheet33"/>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8">
+        <v>7</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E10">
+        <v>9</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="G2:G10" xr:uid="{D9F2857C-EA9E-CB49-9CF8-07047A99E53B}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{422AE880-0C69-104F-AA9B-DA4856BD7616}">
   <sheetPr codeName="Sheet34"/>
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
@@ -8369,7 +8476,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46399228-8395-7647-B644-8C049B767FB1}">
   <sheetPr codeName="Sheet35"/>
   <dimension ref="A1:G6"/>
@@ -8497,7 +8604,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DB5B155-5FF2-2144-9081-38DF5FF7C409}">
   <sheetPr codeName="Sheet36"/>
   <dimension ref="A1:G7"/>

</xml_diff>

<commit_message>
Fix route schedule reload and next-day truck handling
</commit_message>
<xml_diff>
--- a/RouteSchedule.xlsx
+++ b/RouteSchedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marshallhuckins/Desktop/AMS Routes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA00708F-27F0-7E47-BFF3-74D82E75E3DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16195444-1550-E04A-AD6D-E7345D0934ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" firstSheet="27" activeTab="35" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14480" yWindow="680" windowWidth="34200" windowHeight="21460" firstSheet="12" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="21_URBANDALE" sheetId="42" r:id="rId1"/>
@@ -1953,10 +1953,10 @@
         <v>43</v>
       </c>
       <c r="C3" s="2">
+        <v>0.59027777777777779</v>
+      </c>
+      <c r="D3" s="2">
         <v>0.59375</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.63888888888888884</v>
       </c>
       <c r="E3">
         <v>2</v>

</xml_diff>